<commit_message>
Přidej fiktivní data výdejů léků 2026 a report z nich
vytvor_data_leky.py z loňského sešitu vytvoří stejný sešit pro nový rok
(zachová listy, vzorce a formáty). vytvor_report_leky.py nově čte data
ze sešitu místo vlastního generování – na datech 2025 dává report
shodný s report_2025_12.xlsx.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_018ES8jrK8HNw8yf4RQivJNy
</commit_message>
<xml_diff>
--- a/reporty/report_2026_12.xlsx
+++ b/reporty/report_2026_12.xlsx
@@ -547,7 +547,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Zdroj: fiktivní data 2026 (vytvor_report_leky.py) · srovnání s měsícem listopad 2026 · zvýrazněny změny nad ±20%</t>
+          <t>Zdroj: ukazkova_data_leky_pacienti_2026.xlsx · srovnání s měsícem listopad 2026 · zvýrazněny změny nad ±20%</t>
         </is>
       </c>
     </row>
@@ -592,10 +592,10 @@
         </is>
       </c>
       <c r="B6" s="4" t="n">
-        <v>14500</v>
+        <v>10805</v>
       </c>
       <c r="C6" s="4" t="n">
-        <v>13016</v>
+        <v>12059</v>
       </c>
       <c r="D6" s="4">
         <f>B6-C6</f>
@@ -613,10 +613,10 @@
         </is>
       </c>
       <c r="B7" s="4" t="n">
-        <v>115</v>
+        <v>89</v>
       </c>
       <c r="C7" s="4" t="n">
-        <v>109</v>
+        <v>103</v>
       </c>
       <c r="D7" s="4">
         <f>B7-C7</f>
@@ -634,10 +634,10 @@
         </is>
       </c>
       <c r="B8" s="4" t="n">
-        <v>94</v>
+        <v>86</v>
       </c>
       <c r="C8" s="4" t="n">
-        <v>86</v>
+        <v>93</v>
       </c>
       <c r="D8" s="4">
         <f>B8-C8</f>
@@ -655,10 +655,10 @@
         </is>
       </c>
       <c r="B9" s="4" t="n">
-        <v>52</v>
+        <v>55</v>
       </c>
       <c r="C9" s="4" t="n">
-        <v>49</v>
+        <v>53</v>
       </c>
       <c r="D9" s="4">
         <f>B9-C9</f>
@@ -737,14 +737,14 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Sertralin 50 mg</t>
+          <t>Levothyroxin 50 µg</t>
         </is>
       </c>
       <c r="B15" s="4" t="n">
-        <v>3010</v>
+        <v>1708</v>
       </c>
       <c r="C15" s="4" t="n">
-        <v>2795</v>
+        <v>1708</v>
       </c>
       <c r="D15" s="4">
         <f>B15-C15</f>
@@ -758,20 +758,20 @@
         <v>14</v>
       </c>
       <c r="G15" s="4" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Omeprazol 20 mg</t>
+          <t>Ramipril 5 mg</t>
         </is>
       </c>
       <c r="B16" s="4" t="n">
-        <v>2363</v>
+        <v>1515</v>
       </c>
       <c r="C16" s="4" t="n">
-        <v>1529</v>
+        <v>1414</v>
       </c>
       <c r="D16" s="4">
         <f>B16-C16</f>
@@ -782,23 +782,23 @@
         <v/>
       </c>
       <c r="F16" s="4" t="n">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="G16" s="4" t="n">
-        <v>11</v>
+        <v>14</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Atorvastatin 20 mg</t>
+          <t>Sertralin 50 mg</t>
         </is>
       </c>
       <c r="B17" s="4" t="n">
-        <v>1788</v>
+        <v>1512</v>
       </c>
       <c r="C17" s="4" t="n">
-        <v>1639</v>
+        <v>1080</v>
       </c>
       <c r="D17" s="4">
         <f>B17-C17</f>
@@ -809,23 +809,23 @@
         <v/>
       </c>
       <c r="F17" s="4" t="n">
-        <v>12</v>
+        <v>7</v>
       </c>
       <c r="G17" s="4" t="n">
-        <v>11</v>
+        <v>5</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Metformin 500 mg</t>
+          <t>Omeprazol 20 mg</t>
         </is>
       </c>
       <c r="B18" s="4" t="n">
-        <v>1656</v>
+        <v>1251</v>
       </c>
       <c r="C18" s="4" t="n">
-        <v>1380</v>
+        <v>1807</v>
       </c>
       <c r="D18" s="4">
         <f>B18-C18</f>
@@ -836,23 +836,23 @@
         <v/>
       </c>
       <c r="F18" s="4" t="n">
-        <v>18</v>
+        <v>9</v>
       </c>
       <c r="G18" s="4" t="n">
-        <v>15</v>
+        <v>13</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Ramipril 5 mg</t>
+          <t>Salbutamol inhalátor</t>
         </is>
       </c>
       <c r="B19" s="4" t="n">
-        <v>1212</v>
+        <v>1190</v>
       </c>
       <c r="C19" s="4" t="n">
-        <v>1717</v>
+        <v>1020</v>
       </c>
       <c r="D19" s="4">
         <f>B19-C19</f>
@@ -863,23 +863,23 @@
         <v/>
       </c>
       <c r="F19" s="4" t="n">
-        <v>12</v>
+        <v>7</v>
       </c>
       <c r="G19" s="4" t="n">
-        <v>17</v>
+        <v>6</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Amlodipin 5 mg</t>
+          <t>Amoxicilin 500 mg</t>
         </is>
       </c>
       <c r="B20" s="4" t="n">
-        <v>1184</v>
+        <v>992</v>
       </c>
       <c r="C20" s="4" t="n">
-        <v>1258</v>
+        <v>1488</v>
       </c>
       <c r="D20" s="4">
         <f>B20-C20</f>
@@ -890,23 +890,23 @@
         <v/>
       </c>
       <c r="F20" s="4" t="n">
-        <v>16</v>
+        <v>8</v>
       </c>
       <c r="G20" s="4" t="n">
-        <v>17</v>
+        <v>12</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Salbutamol inhalátor</t>
+          <t>Amlodipin 5 mg</t>
         </is>
       </c>
       <c r="B21" s="4" t="n">
-        <v>1183</v>
+        <v>888</v>
       </c>
       <c r="C21" s="4" t="n">
-        <v>338</v>
+        <v>1110</v>
       </c>
       <c r="D21" s="4">
         <f>B21-C21</f>
@@ -917,23 +917,23 @@
         <v/>
       </c>
       <c r="F21" s="4" t="n">
-        <v>7</v>
+        <v>12</v>
       </c>
       <c r="G21" s="4" t="n">
-        <v>2</v>
+        <v>15</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Levothyroxin 50 µg</t>
+          <t>Atorvastatin 20 mg</t>
         </is>
       </c>
       <c r="B22" s="4" t="n">
-        <v>968</v>
+        <v>745</v>
       </c>
       <c r="C22" s="4" t="n">
-        <v>1452</v>
+        <v>1043</v>
       </c>
       <c r="D22" s="4">
         <f>B22-C22</f>
@@ -944,23 +944,23 @@
         <v/>
       </c>
       <c r="F22" s="4" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="G22" s="4" t="n">
-        <v>12</v>
+        <v>7</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Amoxicilin 500 mg</t>
+          <t>Metformin 500 mg</t>
         </is>
       </c>
       <c r="B23" s="4" t="n">
-        <v>868</v>
+        <v>736</v>
       </c>
       <c r="C23" s="4" t="n">
-        <v>372</v>
+        <v>920</v>
       </c>
       <c r="D23" s="4">
         <f>B23-C23</f>
@@ -971,10 +971,10 @@
         <v/>
       </c>
       <c r="F23" s="4" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="G23" s="4" t="n">
-        <v>3</v>
+        <v>10</v>
       </c>
     </row>
     <row r="24">
@@ -987,7 +987,7 @@
         <v>268</v>
       </c>
       <c r="C24" s="4" t="n">
-        <v>536</v>
+        <v>469</v>
       </c>
       <c r="D24" s="4">
         <f>B24-C24</f>
@@ -1001,7 +1001,7 @@
         <v>4</v>
       </c>
       <c r="G24" s="4" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
     </row>
     <row r="25">
@@ -1082,14 +1082,14 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Středočeský</t>
+          <t>Praha</t>
         </is>
       </c>
       <c r="B30" s="4" t="n">
-        <v>5486</v>
+        <v>2862</v>
       </c>
       <c r="C30" s="4" t="n">
-        <v>4575</v>
+        <v>2791</v>
       </c>
       <c r="D30" s="4">
         <f>B30-C30</f>
@@ -1100,10 +1100,10 @@
         <v/>
       </c>
       <c r="F30" s="4" t="n">
-        <v>45</v>
+        <v>23</v>
       </c>
       <c r="G30" s="4" t="n">
-        <v>39</v>
+        <v>26</v>
       </c>
     </row>
     <row r="31">
@@ -1113,10 +1113,10 @@
         </is>
       </c>
       <c r="B31" s="4" t="n">
-        <v>3648</v>
+        <v>2697</v>
       </c>
       <c r="C31" s="4" t="n">
-        <v>3713</v>
+        <v>3311</v>
       </c>
       <c r="D31" s="4">
         <f>B31-C31</f>
@@ -1127,23 +1127,23 @@
         <v/>
       </c>
       <c r="F31" s="4" t="n">
-        <v>27</v>
+        <v>20</v>
       </c>
       <c r="G31" s="4" t="n">
-        <v>30</v>
+        <v>24</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>Moravskoslezský</t>
+          <t>Středočeský</t>
         </is>
       </c>
       <c r="B32" s="4" t="n">
-        <v>1622</v>
+        <v>2566</v>
       </c>
       <c r="C32" s="4" t="n">
-        <v>1878</v>
+        <v>2580</v>
       </c>
       <c r="D32" s="4">
         <f>B32-C32</f>
@@ -1154,23 +1154,23 @@
         <v/>
       </c>
       <c r="F32" s="4" t="n">
-        <v>13</v>
+        <v>22</v>
       </c>
       <c r="G32" s="4" t="n">
-        <v>15</v>
+        <v>22</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Praha</t>
+          <t>Olomoucký</t>
         </is>
       </c>
       <c r="B33" s="4" t="n">
-        <v>1390</v>
+        <v>1029</v>
       </c>
       <c r="C33" s="4" t="n">
-        <v>892</v>
+        <v>1659</v>
       </c>
       <c r="D33" s="4">
         <f>B33-C33</f>
@@ -1181,10 +1181,10 @@
         <v/>
       </c>
       <c r="F33" s="4" t="n">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="G33" s="4" t="n">
-        <v>9</v>
+        <v>15</v>
       </c>
     </row>
     <row r="34">
@@ -1194,10 +1194,10 @@
         </is>
       </c>
       <c r="B34" s="4" t="n">
-        <v>1229</v>
+        <v>954</v>
       </c>
       <c r="C34" s="4" t="n">
-        <v>1288</v>
+        <v>1103</v>
       </c>
       <c r="D34" s="4">
         <f>B34-C34</f>
@@ -1208,23 +1208,23 @@
         <v/>
       </c>
       <c r="F34" s="4" t="n">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="G34" s="4" t="n">
-        <v>12</v>
+        <v>10</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>Olomoucký</t>
+          <t>Moravskoslezský</t>
         </is>
       </c>
       <c r="B35" s="4" t="n">
-        <v>1125</v>
+        <v>697</v>
       </c>
       <c r="C35" s="4" t="n">
-        <v>670</v>
+        <v>615</v>
       </c>
       <c r="D35" s="4">
         <f>B35-C35</f>
@@ -1235,10 +1235,10 @@
         <v/>
       </c>
       <c r="F35" s="4" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="G35" s="4" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
     </row>
     <row r="36">
@@ -1329,7 +1329,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H95"/>
+  <dimension ref="A1:H87"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -1395,27 +1395,27 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Praha</t>
+          <t>Středočeský</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>L05</t>
+          <t>L01</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Levothyroxin 50 µg</t>
+          <t>Metformin 500 mg</t>
         </is>
       </c>
       <c r="F2" t="n">
         <v>1</v>
       </c>
       <c r="G2" t="n">
-        <v>121</v>
+        <v>92</v>
       </c>
       <c r="H2" t="n">
-        <v>121</v>
+        <v>92</v>
       </c>
     </row>
     <row r="3">
@@ -1429,27 +1429,27 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Jihomoravský</t>
+          <t>Olomoucký</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>L03</t>
+          <t>L09</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Amlodipin 5 mg</t>
+          <t>Amoxicilin 500 mg</t>
         </is>
       </c>
       <c r="F3" t="n">
         <v>1</v>
       </c>
       <c r="G3" t="n">
-        <v>74</v>
+        <v>124</v>
       </c>
       <c r="H3" t="n">
-        <v>74</v>
+        <v>124</v>
       </c>
     </row>
     <row r="4">
@@ -1458,12 +1458,12 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>P0002</t>
+          <t>P0003</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Jihomoravský</t>
+          <t>Praha</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -1497,27 +1497,27 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Středočeský</t>
+          <t>Praha</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>L06</t>
+          <t>L09</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Omeprazol 20 mg</t>
+          <t>Amoxicilin 500 mg</t>
         </is>
       </c>
       <c r="F5" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G5" t="n">
-        <v>139</v>
+        <v>124</v>
       </c>
       <c r="H5" t="n">
-        <v>278</v>
+        <v>124</v>
       </c>
     </row>
     <row r="6">
@@ -1526,32 +1526,32 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>P0003</t>
+          <t>P0004</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Středočeský</t>
+          <t>Jihomoravský</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>L08</t>
+          <t>L04</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Salbutamol inhalátor</t>
+          <t>Ramipril 5 mg</t>
         </is>
       </c>
       <c r="F6" t="n">
         <v>1</v>
       </c>
       <c r="G6" t="n">
-        <v>169</v>
+        <v>101</v>
       </c>
       <c r="H6" t="n">
-        <v>169</v>
+        <v>101</v>
       </c>
     </row>
     <row r="7">
@@ -1560,7 +1560,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>P0004</t>
+          <t>P0005</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -1570,22 +1570,22 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>L03</t>
+          <t>L09</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Amlodipin 5 mg</t>
+          <t>Amoxicilin 500 mg</t>
         </is>
       </c>
       <c r="F7" t="n">
         <v>1</v>
       </c>
       <c r="G7" t="n">
-        <v>74</v>
+        <v>124</v>
       </c>
       <c r="H7" t="n">
-        <v>74</v>
+        <v>124</v>
       </c>
     </row>
     <row r="8">
@@ -1594,32 +1594,32 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>P0004</t>
+          <t>P0006</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Středočeský</t>
+          <t>Jihomoravský</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>L05</t>
+          <t>L03</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Levothyroxin 50 µg</t>
+          <t>Amlodipin 5 mg</t>
         </is>
       </c>
       <c r="F8" t="n">
         <v>1</v>
       </c>
       <c r="G8" t="n">
-        <v>121</v>
+        <v>74</v>
       </c>
       <c r="H8" t="n">
-        <v>121</v>
+        <v>74</v>
       </c>
     </row>
     <row r="9">
@@ -1628,32 +1628,32 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>P0004</t>
+          <t>P0008</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Středočeský</t>
+          <t>Jihomoravský</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>L07</t>
+          <t>L08</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Sertralin 50 mg</t>
+          <t>Salbutamol inhalátor</t>
         </is>
       </c>
       <c r="F9" t="n">
         <v>1</v>
       </c>
       <c r="G9" t="n">
-        <v>215</v>
+        <v>170</v>
       </c>
       <c r="H9" t="n">
-        <v>215</v>
+        <v>170</v>
       </c>
     </row>
     <row r="10">
@@ -1662,32 +1662,32 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>P0005</t>
+          <t>P0009</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Středočeský</t>
+          <t>Praha</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>L01</t>
+          <t>L08</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Metformin 500 mg</t>
+          <t>Salbutamol inhalátor</t>
         </is>
       </c>
       <c r="F10" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G10" t="n">
-        <v>92</v>
+        <v>170</v>
       </c>
       <c r="H10" t="n">
-        <v>184</v>
+        <v>170</v>
       </c>
     </row>
     <row r="11">
@@ -1696,32 +1696,32 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>P0006</t>
+          <t>P0009</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Plzeňský</t>
+          <t>Praha</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>L07</t>
+          <t>L09</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Sertralin 50 mg</t>
+          <t>Amoxicilin 500 mg</t>
         </is>
       </c>
       <c r="F11" t="n">
         <v>1</v>
       </c>
       <c r="G11" t="n">
-        <v>215</v>
+        <v>124</v>
       </c>
       <c r="H11" t="n">
-        <v>215</v>
+        <v>124</v>
       </c>
     </row>
     <row r="12">
@@ -1730,12 +1730,12 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>P0007</t>
+          <t>P0011</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Moravskoslezský</t>
+          <t>Olomoucký</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
@@ -1749,13 +1749,13 @@
         </is>
       </c>
       <c r="F12" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G12" t="n">
         <v>74</v>
       </c>
       <c r="H12" t="n">
-        <v>148</v>
+        <v>74</v>
       </c>
     </row>
     <row r="13">
@@ -1764,7 +1764,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>P0007</t>
+          <t>P0012</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -1774,22 +1774,22 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>L06</t>
+          <t>L07</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>Omeprazol 20 mg</t>
+          <t>Sertralin 50 mg</t>
         </is>
       </c>
       <c r="F13" t="n">
         <v>1</v>
       </c>
       <c r="G13" t="n">
-        <v>139</v>
+        <v>216</v>
       </c>
       <c r="H13" t="n">
-        <v>139</v>
+        <v>216</v>
       </c>
     </row>
     <row r="14">
@@ -1798,32 +1798,32 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>P0008</t>
+          <t>P0014</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Praha</t>
+          <t>Moravskoslezský</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>L03</t>
+          <t>L04</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>Amlodipin 5 mg</t>
+          <t>Ramipril 5 mg</t>
         </is>
       </c>
       <c r="F14" t="n">
         <v>1</v>
       </c>
       <c r="G14" t="n">
-        <v>74</v>
+        <v>101</v>
       </c>
       <c r="H14" t="n">
-        <v>74</v>
+        <v>101</v>
       </c>
     </row>
     <row r="15">
@@ -1832,7 +1832,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>P0009</t>
+          <t>P0015</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -1842,22 +1842,22 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>L03</t>
+          <t>L01</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>Amlodipin 5 mg</t>
+          <t>Metformin 500 mg</t>
         </is>
       </c>
       <c r="F15" t="n">
         <v>1</v>
       </c>
       <c r="G15" t="n">
-        <v>74</v>
+        <v>92</v>
       </c>
       <c r="H15" t="n">
-        <v>74</v>
+        <v>92</v>
       </c>
     </row>
     <row r="16">
@@ -1866,7 +1866,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>P0009</t>
+          <t>P0015</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -1876,22 +1876,22 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>L04</t>
+          <t>L07</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>Ramipril 5 mg</t>
+          <t>Sertralin 50 mg</t>
         </is>
       </c>
       <c r="F16" t="n">
         <v>1</v>
       </c>
       <c r="G16" t="n">
-        <v>101</v>
+        <v>216</v>
       </c>
       <c r="H16" t="n">
-        <v>101</v>
+        <v>216</v>
       </c>
     </row>
     <row r="17">
@@ -1900,12 +1900,12 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>P0009</t>
+          <t>P0016</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Jihomoravský</t>
+          <t>Středočeský</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
@@ -1919,13 +1919,13 @@
         </is>
       </c>
       <c r="F17" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G17" t="n">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="H17" t="n">
-        <v>121</v>
+        <v>244</v>
       </c>
     </row>
     <row r="18">
@@ -1934,32 +1934,32 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>P0010</t>
+          <t>P0017</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Středočeský</t>
+          <t>Plzeňský</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>L02</t>
+          <t>L01</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>Atorvastatin 20 mg</t>
+          <t>Metformin 500 mg</t>
         </is>
       </c>
       <c r="F18" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G18" t="n">
-        <v>149</v>
+        <v>92</v>
       </c>
       <c r="H18" t="n">
-        <v>298</v>
+        <v>92</v>
       </c>
     </row>
     <row r="19">
@@ -1968,32 +1968,32 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>P0010</t>
+          <t>P0017</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Středočeský</t>
+          <t>Plzeňský</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>L03</t>
+          <t>L04</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>Amlodipin 5 mg</t>
+          <t>Ramipril 5 mg</t>
         </is>
       </c>
       <c r="F19" t="n">
         <v>1</v>
       </c>
       <c r="G19" t="n">
-        <v>74</v>
+        <v>101</v>
       </c>
       <c r="H19" t="n">
-        <v>74</v>
+        <v>101</v>
       </c>
     </row>
     <row r="20">
@@ -2002,12 +2002,12 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>P0011</t>
+          <t>P0017</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Olomoucký</t>
+          <t>Plzeňský</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
@@ -2036,32 +2036,32 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>P0011</t>
+          <t>P0018</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Olomoucký</t>
+          <t>Praha</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>L07</t>
+          <t>L03</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>Sertralin 50 mg</t>
+          <t>Amlodipin 5 mg</t>
         </is>
       </c>
       <c r="F21" t="n">
         <v>1</v>
       </c>
       <c r="G21" t="n">
-        <v>215</v>
+        <v>74</v>
       </c>
       <c r="H21" t="n">
-        <v>215</v>
+        <v>74</v>
       </c>
     </row>
     <row r="22">
@@ -2070,12 +2070,12 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>P0012</t>
+          <t>P0018</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Moravskoslezský</t>
+          <t>Praha</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
@@ -2089,13 +2089,13 @@
         </is>
       </c>
       <c r="F22" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G22" t="n">
-        <v>215</v>
+        <v>216</v>
       </c>
       <c r="H22" t="n">
-        <v>430</v>
+        <v>216</v>
       </c>
     </row>
     <row r="23">
@@ -2104,32 +2104,32 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>P0013</t>
+          <t>P0019</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Jihomoravský</t>
+          <t>Plzeňský</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>L01</t>
+          <t>L04</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>Metformin 500 mg</t>
+          <t>Ramipril 5 mg</t>
         </is>
       </c>
       <c r="F23" t="n">
         <v>1</v>
       </c>
       <c r="G23" t="n">
-        <v>92</v>
+        <v>101</v>
       </c>
       <c r="H23" t="n">
-        <v>92</v>
+        <v>101</v>
       </c>
     </row>
     <row r="24">
@@ -2138,32 +2138,32 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>P0013</t>
+          <t>P0019</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Jihomoravský</t>
+          <t>Plzeňský</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>L09</t>
+          <t>L10</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>Amoxicilin 500 mg</t>
+          <t>Ibuprofen 400 mg</t>
         </is>
       </c>
       <c r="F24" t="n">
         <v>1</v>
       </c>
       <c r="G24" t="n">
-        <v>124</v>
+        <v>67</v>
       </c>
       <c r="H24" t="n">
-        <v>124</v>
+        <v>67</v>
       </c>
     </row>
     <row r="25">
@@ -2172,7 +2172,7 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>P0014</t>
+          <t>P0021</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
@@ -2182,22 +2182,22 @@
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>L10</t>
+          <t>L01</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>Ibuprofen 400 mg</t>
+          <t>Metformin 500 mg</t>
         </is>
       </c>
       <c r="F25" t="n">
         <v>1</v>
       </c>
       <c r="G25" t="n">
-        <v>67</v>
+        <v>92</v>
       </c>
       <c r="H25" t="n">
-        <v>67</v>
+        <v>92</v>
       </c>
     </row>
     <row r="26">
@@ -2206,7 +2206,7 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>P0015</t>
+          <t>P0022</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
@@ -2216,22 +2216,22 @@
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>L02</t>
+          <t>L07</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>Atorvastatin 20 mg</t>
+          <t>Sertralin 50 mg</t>
         </is>
       </c>
       <c r="F26" t="n">
         <v>1</v>
       </c>
       <c r="G26" t="n">
-        <v>149</v>
+        <v>216</v>
       </c>
       <c r="H26" t="n">
-        <v>149</v>
+        <v>216</v>
       </c>
     </row>
     <row r="27">
@@ -2240,32 +2240,32 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>P0016</t>
+          <t>P0023</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Moravskoslezský</t>
+          <t>Středočeský</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>L01</t>
+          <t>L03</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>Metformin 500 mg</t>
+          <t>Amlodipin 5 mg</t>
         </is>
       </c>
       <c r="F27" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G27" t="n">
-        <v>92</v>
+        <v>74</v>
       </c>
       <c r="H27" t="n">
-        <v>184</v>
+        <v>74</v>
       </c>
     </row>
     <row r="28">
@@ -2274,32 +2274,32 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>P0016</t>
+          <t>P0023</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>Moravskoslezský</t>
+          <t>Středočeský</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>L08</t>
+          <t>L05</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>Salbutamol inhalátor</t>
+          <t>Levothyroxin 50 µg</t>
         </is>
       </c>
       <c r="F28" t="n">
         <v>1</v>
       </c>
       <c r="G28" t="n">
-        <v>169</v>
+        <v>122</v>
       </c>
       <c r="H28" t="n">
-        <v>169</v>
+        <v>122</v>
       </c>
     </row>
     <row r="29">
@@ -2308,32 +2308,32 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>P0016</t>
+          <t>P0023</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Moravskoslezský</t>
+          <t>Středočeský</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>L09</t>
+          <t>L06</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>Amoxicilin 500 mg</t>
+          <t>Omeprazol 20 mg</t>
         </is>
       </c>
       <c r="F29" t="n">
         <v>1</v>
       </c>
       <c r="G29" t="n">
-        <v>124</v>
+        <v>139</v>
       </c>
       <c r="H29" t="n">
-        <v>124</v>
+        <v>139</v>
       </c>
     </row>
     <row r="30">
@@ -2342,32 +2342,32 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>P0016</t>
+          <t>P0024</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Moravskoslezský</t>
+          <t>Jihomoravský</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>L10</t>
+          <t>L08</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>Ibuprofen 400 mg</t>
+          <t>Salbutamol inhalátor</t>
         </is>
       </c>
       <c r="F30" t="n">
         <v>1</v>
       </c>
       <c r="G30" t="n">
-        <v>67</v>
+        <v>170</v>
       </c>
       <c r="H30" t="n">
-        <v>67</v>
+        <v>170</v>
       </c>
     </row>
     <row r="31">
@@ -2376,32 +2376,32 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>P0017</t>
+          <t>P0025</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Středočeský</t>
+          <t>Olomoucký</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>L01</t>
+          <t>L03</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>Metformin 500 mg</t>
+          <t>Amlodipin 5 mg</t>
         </is>
       </c>
       <c r="F31" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G31" t="n">
-        <v>92</v>
+        <v>74</v>
       </c>
       <c r="H31" t="n">
-        <v>184</v>
+        <v>74</v>
       </c>
     </row>
     <row r="32">
@@ -2410,32 +2410,32 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>P0017</t>
+          <t>P0026</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>Středočeský</t>
+          <t>Jihomoravský</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>L06</t>
+          <t>L04</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>Omeprazol 20 mg</t>
+          <t>Ramipril 5 mg</t>
         </is>
       </c>
       <c r="F32" t="n">
         <v>1</v>
       </c>
       <c r="G32" t="n">
-        <v>139</v>
+        <v>101</v>
       </c>
       <c r="H32" t="n">
-        <v>139</v>
+        <v>101</v>
       </c>
     </row>
     <row r="33">
@@ -2444,32 +2444,32 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>P0018</t>
+          <t>P0026</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>Středočeský</t>
+          <t>Jihomoravský</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>L03</t>
+          <t>L08</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>Amlodipin 5 mg</t>
+          <t>Salbutamol inhalátor</t>
         </is>
       </c>
       <c r="F33" t="n">
         <v>1</v>
       </c>
       <c r="G33" t="n">
-        <v>74</v>
+        <v>170</v>
       </c>
       <c r="H33" t="n">
-        <v>74</v>
+        <v>170</v>
       </c>
     </row>
     <row r="34">
@@ -2478,12 +2478,12 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>P0019</t>
+          <t>P0027</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>Středočeský</t>
+          <t>Jihomoravský</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
@@ -2512,32 +2512,32 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>P0019</t>
+          <t>P0030</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>Středočeský</t>
+          <t>Jihomoravský</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>L06</t>
+          <t>L02</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>Omeprazol 20 mg</t>
+          <t>Atorvastatin 20 mg</t>
         </is>
       </c>
       <c r="F35" t="n">
         <v>1</v>
       </c>
       <c r="G35" t="n">
-        <v>139</v>
+        <v>149</v>
       </c>
       <c r="H35" t="n">
-        <v>139</v>
+        <v>149</v>
       </c>
     </row>
     <row r="36">
@@ -2546,32 +2546,32 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>P0019</t>
+          <t>P0030</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>Středočeský</t>
+          <t>Jihomoravský</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>L08</t>
+          <t>L05</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>Salbutamol inhalátor</t>
+          <t>Levothyroxin 50 µg</t>
         </is>
       </c>
       <c r="F36" t="n">
         <v>1</v>
       </c>
       <c r="G36" t="n">
-        <v>169</v>
+        <v>122</v>
       </c>
       <c r="H36" t="n">
-        <v>169</v>
+        <v>122</v>
       </c>
     </row>
     <row r="37">
@@ -2580,7 +2580,7 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>P0021</t>
+          <t>P0031</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
@@ -2590,22 +2590,22 @@
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>L07</t>
+          <t>L10</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>Sertralin 50 mg</t>
+          <t>Ibuprofen 400 mg</t>
         </is>
       </c>
       <c r="F37" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G37" t="n">
-        <v>215</v>
+        <v>67</v>
       </c>
       <c r="H37" t="n">
-        <v>430</v>
+        <v>67</v>
       </c>
     </row>
     <row r="38">
@@ -2614,12 +2614,12 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>P0023</t>
+          <t>P0032</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>Jihomoravský</t>
+          <t>Praha</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
@@ -2633,13 +2633,13 @@
         </is>
       </c>
       <c r="F38" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G38" t="n">
         <v>92</v>
       </c>
       <c r="H38" t="n">
-        <v>184</v>
+        <v>92</v>
       </c>
     </row>
     <row r="39">
@@ -2648,32 +2648,32 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>P0023</t>
+          <t>P0033</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>Jihomoravský</t>
+          <t>Praha</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>L04</t>
+          <t>L10</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>Ramipril 5 mg</t>
+          <t>Ibuprofen 400 mg</t>
         </is>
       </c>
       <c r="F39" t="n">
         <v>1</v>
       </c>
       <c r="G39" t="n">
-        <v>101</v>
+        <v>67</v>
       </c>
       <c r="H39" t="n">
-        <v>101</v>
+        <v>67</v>
       </c>
     </row>
     <row r="40">
@@ -2682,7 +2682,7 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>P0023</t>
+          <t>P0034</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
@@ -2692,22 +2692,22 @@
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>L08</t>
+          <t>L03</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>Salbutamol inhalátor</t>
+          <t>Amlodipin 5 mg</t>
         </is>
       </c>
       <c r="F40" t="n">
         <v>1</v>
       </c>
       <c r="G40" t="n">
-        <v>169</v>
+        <v>74</v>
       </c>
       <c r="H40" t="n">
-        <v>169</v>
+        <v>74</v>
       </c>
     </row>
     <row r="41">
@@ -2716,12 +2716,12 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>P0024</t>
+          <t>P0035</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>Praha</t>
+          <t>Plzeňský</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
@@ -2750,32 +2750,32 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>P0024</t>
+          <t>P0035</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>Praha</t>
+          <t>Plzeňský</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>L09</t>
+          <t>L05</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>Amoxicilin 500 mg</t>
+          <t>Levothyroxin 50 µg</t>
         </is>
       </c>
       <c r="F42" t="n">
         <v>1</v>
       </c>
       <c r="G42" t="n">
-        <v>124</v>
+        <v>122</v>
       </c>
       <c r="H42" t="n">
-        <v>124</v>
+        <v>122</v>
       </c>
     </row>
     <row r="43">
@@ -2784,32 +2784,32 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>P0025</t>
+          <t>P0036</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>Středočeský</t>
+          <t>Plzeňský</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>L02</t>
+          <t>L06</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>Atorvastatin 20 mg</t>
+          <t>Omeprazol 20 mg</t>
         </is>
       </c>
       <c r="F43" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G43" t="n">
-        <v>149</v>
+        <v>139</v>
       </c>
       <c r="H43" t="n">
-        <v>298</v>
+        <v>139</v>
       </c>
     </row>
     <row r="44">
@@ -2818,7 +2818,7 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>P0025</t>
+          <t>P0037</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
@@ -2828,22 +2828,22 @@
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>L06</t>
+          <t>L04</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>Omeprazol 20 mg</t>
+          <t>Ramipril 5 mg</t>
         </is>
       </c>
       <c r="F44" t="n">
         <v>1</v>
       </c>
       <c r="G44" t="n">
-        <v>139</v>
+        <v>101</v>
       </c>
       <c r="H44" t="n">
-        <v>139</v>
+        <v>101</v>
       </c>
     </row>
     <row r="45">
@@ -2852,7 +2852,7 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>P0026</t>
+          <t>P0037</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
@@ -2862,22 +2862,22 @@
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>L01</t>
+          <t>L08</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>Metformin 500 mg</t>
+          <t>Salbutamol inhalátor</t>
         </is>
       </c>
       <c r="F45" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G45" t="n">
-        <v>92</v>
+        <v>170</v>
       </c>
       <c r="H45" t="n">
-        <v>184</v>
+        <v>170</v>
       </c>
     </row>
     <row r="46">
@@ -2886,12 +2886,12 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>P0026</t>
+          <t>P0039</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>Středočeský</t>
+          <t>Praha</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
@@ -2920,7 +2920,7 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>P0026</t>
+          <t>P0040</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
@@ -2930,22 +2930,22 @@
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>L05</t>
+          <t>L02</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>Levothyroxin 50 µg</t>
+          <t>Atorvastatin 20 mg</t>
         </is>
       </c>
       <c r="F47" t="n">
         <v>1</v>
       </c>
       <c r="G47" t="n">
-        <v>121</v>
+        <v>149</v>
       </c>
       <c r="H47" t="n">
-        <v>121</v>
+        <v>149</v>
       </c>
     </row>
     <row r="48">
@@ -2954,7 +2954,7 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>P0026</t>
+          <t>P0040</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
@@ -2964,22 +2964,22 @@
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>L08</t>
+          <t>L03</t>
         </is>
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>Salbutamol inhalátor</t>
+          <t>Amlodipin 5 mg</t>
         </is>
       </c>
       <c r="F48" t="n">
         <v>1</v>
       </c>
       <c r="G48" t="n">
-        <v>169</v>
+        <v>74</v>
       </c>
       <c r="H48" t="n">
-        <v>169</v>
+        <v>74</v>
       </c>
     </row>
     <row r="49">
@@ -2988,7 +2988,7 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>P0026</t>
+          <t>P0040</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
@@ -2998,22 +2998,22 @@
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>L10</t>
+          <t>L09</t>
         </is>
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>Ibuprofen 400 mg</t>
+          <t>Amoxicilin 500 mg</t>
         </is>
       </c>
       <c r="F49" t="n">
         <v>1</v>
       </c>
       <c r="G49" t="n">
-        <v>67</v>
+        <v>124</v>
       </c>
       <c r="H49" t="n">
-        <v>67</v>
+        <v>124</v>
       </c>
     </row>
     <row r="50">
@@ -3022,32 +3022,32 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>P0027</t>
+          <t>P0041</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>Praha</t>
+          <t>Středočeský</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>L09</t>
+          <t>L02</t>
         </is>
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>Amoxicilin 500 mg</t>
+          <t>Atorvastatin 20 mg</t>
         </is>
       </c>
       <c r="F50" t="n">
         <v>1</v>
       </c>
       <c r="G50" t="n">
-        <v>124</v>
+        <v>149</v>
       </c>
       <c r="H50" t="n">
-        <v>124</v>
+        <v>149</v>
       </c>
     </row>
     <row r="51">
@@ -3056,7 +3056,7 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>P0029</t>
+          <t>P0041</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
@@ -3066,22 +3066,22 @@
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>L01</t>
+          <t>L04</t>
         </is>
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>Metformin 500 mg</t>
+          <t>Ramipril 5 mg</t>
         </is>
       </c>
       <c r="F51" t="n">
         <v>1</v>
       </c>
       <c r="G51" t="n">
-        <v>92</v>
+        <v>101</v>
       </c>
       <c r="H51" t="n">
-        <v>92</v>
+        <v>101</v>
       </c>
     </row>
     <row r="52">
@@ -3090,7 +3090,7 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>P0029</t>
+          <t>P0041</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
@@ -3100,22 +3100,22 @@
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>L08</t>
+          <t>L06</t>
         </is>
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>Salbutamol inhalátor</t>
+          <t>Omeprazol 20 mg</t>
         </is>
       </c>
       <c r="F52" t="n">
         <v>1</v>
       </c>
       <c r="G52" t="n">
-        <v>169</v>
+        <v>139</v>
       </c>
       <c r="H52" t="n">
-        <v>169</v>
+        <v>139</v>
       </c>
     </row>
     <row r="53">
@@ -3124,32 +3124,32 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>P0029</t>
+          <t>P0042</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>Středočeský</t>
+          <t>Praha</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>L09</t>
+          <t>L02</t>
         </is>
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>Amoxicilin 500 mg</t>
+          <t>Atorvastatin 20 mg</t>
         </is>
       </c>
       <c r="F53" t="n">
         <v>1</v>
       </c>
       <c r="G53" t="n">
-        <v>124</v>
+        <v>149</v>
       </c>
       <c r="H53" t="n">
-        <v>124</v>
+        <v>149</v>
       </c>
     </row>
     <row r="54">
@@ -3158,32 +3158,32 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>P0029</t>
+          <t>P0042</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>Středočeský</t>
+          <t>Praha</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>L10</t>
+          <t>L05</t>
         </is>
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>Ibuprofen 400 mg</t>
+          <t>Levothyroxin 50 µg</t>
         </is>
       </c>
       <c r="F54" t="n">
         <v>1</v>
       </c>
       <c r="G54" t="n">
-        <v>67</v>
+        <v>122</v>
       </c>
       <c r="H54" t="n">
-        <v>67</v>
+        <v>122</v>
       </c>
     </row>
     <row r="55">
@@ -3192,32 +3192,32 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>P0030</t>
+          <t>P0043</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>Středočeský</t>
+          <t>Praha</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>L06</t>
+          <t>L09</t>
         </is>
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>Omeprazol 20 mg</t>
+          <t>Amoxicilin 500 mg</t>
         </is>
       </c>
       <c r="F55" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G55" t="n">
-        <v>139</v>
+        <v>124</v>
       </c>
       <c r="H55" t="n">
-        <v>278</v>
+        <v>124</v>
       </c>
     </row>
     <row r="56">
@@ -3226,12 +3226,12 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>P0031</t>
+          <t>P0044</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>Praha</t>
+          <t>Jihomoravský</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
@@ -3248,10 +3248,10 @@
         <v>1</v>
       </c>
       <c r="G56" t="n">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="H56" t="n">
-        <v>121</v>
+        <v>122</v>
       </c>
     </row>
     <row r="57">
@@ -3260,32 +3260,32 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>P0031</t>
+          <t>P0045</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>Praha</t>
+          <t>Středočeský</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>L09</t>
+          <t>L03</t>
         </is>
       </c>
       <c r="E57" t="inlineStr">
         <is>
-          <t>Amoxicilin 500 mg</t>
+          <t>Amlodipin 5 mg</t>
         </is>
       </c>
       <c r="F57" t="n">
         <v>1</v>
       </c>
       <c r="G57" t="n">
-        <v>124</v>
+        <v>74</v>
       </c>
       <c r="H57" t="n">
-        <v>124</v>
+        <v>74</v>
       </c>
     </row>
     <row r="58">
@@ -3294,12 +3294,12 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>P0032</t>
+          <t>P0045</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>Moravskoslezský</t>
+          <t>Středočeský</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
@@ -3313,13 +3313,13 @@
         </is>
       </c>
       <c r="F58" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G58" t="n">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="H58" t="n">
-        <v>121</v>
+        <v>244</v>
       </c>
     </row>
     <row r="59">
@@ -3328,32 +3328,32 @@
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>P0032</t>
+          <t>P0046</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>Moravskoslezský</t>
+          <t>Praha</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>L06</t>
+          <t>L01</t>
         </is>
       </c>
       <c r="E59" t="inlineStr">
         <is>
-          <t>Omeprazol 20 mg</t>
+          <t>Metformin 500 mg</t>
         </is>
       </c>
       <c r="F59" t="n">
         <v>1</v>
       </c>
       <c r="G59" t="n">
-        <v>139</v>
+        <v>92</v>
       </c>
       <c r="H59" t="n">
-        <v>139</v>
+        <v>92</v>
       </c>
     </row>
     <row r="60">
@@ -3362,32 +3362,32 @@
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>P0033</t>
+          <t>P0046</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>Plzeňský</t>
+          <t>Praha</t>
         </is>
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>L03</t>
+          <t>L04</t>
         </is>
       </c>
       <c r="E60" t="inlineStr">
         <is>
-          <t>Amlodipin 5 mg</t>
+          <t>Ramipril 5 mg</t>
         </is>
       </c>
       <c r="F60" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G60" t="n">
-        <v>74</v>
+        <v>101</v>
       </c>
       <c r="H60" t="n">
-        <v>148</v>
+        <v>101</v>
       </c>
     </row>
     <row r="61">
@@ -3396,32 +3396,32 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>P0034</t>
+          <t>P0046</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>Jihomoravský</t>
+          <t>Praha</t>
         </is>
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>L01</t>
+          <t>L05</t>
         </is>
       </c>
       <c r="E61" t="inlineStr">
         <is>
-          <t>Metformin 500 mg</t>
+          <t>Levothyroxin 50 µg</t>
         </is>
       </c>
       <c r="F61" t="n">
         <v>1</v>
       </c>
       <c r="G61" t="n">
-        <v>92</v>
+        <v>122</v>
       </c>
       <c r="H61" t="n">
-        <v>92</v>
+        <v>122</v>
       </c>
     </row>
     <row r="62">
@@ -3430,32 +3430,32 @@
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>P0034</t>
+          <t>P0047</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>Jihomoravský</t>
+          <t>Moravskoslezský</t>
         </is>
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>L07</t>
+          <t>L02</t>
         </is>
       </c>
       <c r="E62" t="inlineStr">
         <is>
-          <t>Sertralin 50 mg</t>
+          <t>Atorvastatin 20 mg</t>
         </is>
       </c>
       <c r="F62" t="n">
         <v>1</v>
       </c>
       <c r="G62" t="n">
-        <v>215</v>
+        <v>149</v>
       </c>
       <c r="H62" t="n">
-        <v>215</v>
+        <v>149</v>
       </c>
     </row>
     <row r="63">
@@ -3464,7 +3464,7 @@
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>P0035</t>
+          <t>P0048</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
@@ -3474,22 +3474,22 @@
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>L02</t>
+          <t>L06</t>
         </is>
       </c>
       <c r="E63" t="inlineStr">
         <is>
-          <t>Atorvastatin 20 mg</t>
+          <t>Omeprazol 20 mg</t>
         </is>
       </c>
       <c r="F63" t="n">
         <v>1</v>
       </c>
       <c r="G63" t="n">
-        <v>149</v>
+        <v>139</v>
       </c>
       <c r="H63" t="n">
-        <v>149</v>
+        <v>139</v>
       </c>
     </row>
     <row r="64">
@@ -3498,32 +3498,32 @@
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>P0036</t>
+          <t>P0048</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>Olomoucký</t>
+          <t>Středočeský</t>
         </is>
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>L04</t>
+          <t>L10</t>
         </is>
       </c>
       <c r="E64" t="inlineStr">
         <is>
-          <t>Ramipril 5 mg</t>
+          <t>Ibuprofen 400 mg</t>
         </is>
       </c>
       <c r="F64" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G64" t="n">
-        <v>101</v>
+        <v>67</v>
       </c>
       <c r="H64" t="n">
-        <v>202</v>
+        <v>67</v>
       </c>
     </row>
     <row r="65">
@@ -3532,7 +3532,7 @@
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>P0036</t>
+          <t>P0051</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
@@ -3542,22 +3542,22 @@
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>L06</t>
+          <t>L05</t>
         </is>
       </c>
       <c r="E65" t="inlineStr">
         <is>
-          <t>Omeprazol 20 mg</t>
+          <t>Levothyroxin 50 µg</t>
         </is>
       </c>
       <c r="F65" t="n">
         <v>1</v>
       </c>
       <c r="G65" t="n">
-        <v>139</v>
+        <v>122</v>
       </c>
       <c r="H65" t="n">
-        <v>139</v>
+        <v>122</v>
       </c>
     </row>
     <row r="66">
@@ -3566,32 +3566,32 @@
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>P0036</t>
+          <t>P0052</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>Olomoucký</t>
+          <t>Středočeský</t>
         </is>
       </c>
       <c r="D66" t="inlineStr">
         <is>
-          <t>L07</t>
+          <t>L04</t>
         </is>
       </c>
       <c r="E66" t="inlineStr">
         <is>
-          <t>Sertralin 50 mg</t>
+          <t>Ramipril 5 mg</t>
         </is>
       </c>
       <c r="F66" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G66" t="n">
-        <v>215</v>
+        <v>101</v>
       </c>
       <c r="H66" t="n">
-        <v>430</v>
+        <v>101</v>
       </c>
     </row>
     <row r="67">
@@ -3600,32 +3600,32 @@
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>P0037</t>
+          <t>P0053</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>Jihomoravský</t>
+          <t>Moravskoslezský</t>
         </is>
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>L02</t>
+          <t>L01</t>
         </is>
       </c>
       <c r="E67" t="inlineStr">
         <is>
-          <t>Atorvastatin 20 mg</t>
+          <t>Metformin 500 mg</t>
         </is>
       </c>
       <c r="F67" t="n">
         <v>1</v>
       </c>
       <c r="G67" t="n">
-        <v>149</v>
+        <v>92</v>
       </c>
       <c r="H67" t="n">
-        <v>149</v>
+        <v>92</v>
       </c>
     </row>
     <row r="68">
@@ -3634,32 +3634,32 @@
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>P0037</t>
+          <t>P0055</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>Jihomoravský</t>
+          <t>Středočeský</t>
         </is>
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>L08</t>
+          <t>L06</t>
         </is>
       </c>
       <c r="E68" t="inlineStr">
         <is>
-          <t>Salbutamol inhalátor</t>
+          <t>Omeprazol 20 mg</t>
         </is>
       </c>
       <c r="F68" t="n">
         <v>1</v>
       </c>
       <c r="G68" t="n">
-        <v>169</v>
+        <v>139</v>
       </c>
       <c r="H68" t="n">
-        <v>169</v>
+        <v>139</v>
       </c>
     </row>
     <row r="69">
@@ -3668,32 +3668,32 @@
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>P0038</t>
+          <t>P0056</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>Středočeský</t>
+          <t>Olomoucký</t>
         </is>
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>L03</t>
+          <t>L01</t>
         </is>
       </c>
       <c r="E69" t="inlineStr">
         <is>
-          <t>Amlodipin 5 mg</t>
+          <t>Metformin 500 mg</t>
         </is>
       </c>
       <c r="F69" t="n">
         <v>1</v>
       </c>
       <c r="G69" t="n">
-        <v>74</v>
+        <v>92</v>
       </c>
       <c r="H69" t="n">
-        <v>74</v>
+        <v>92</v>
       </c>
     </row>
     <row r="70">
@@ -3702,32 +3702,32 @@
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>P0039</t>
+          <t>P0056</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>Moravskoslezský</t>
+          <t>Olomoucký</t>
         </is>
       </c>
       <c r="D70" t="inlineStr">
         <is>
-          <t>L04</t>
+          <t>L03</t>
         </is>
       </c>
       <c r="E70" t="inlineStr">
         <is>
-          <t>Ramipril 5 mg</t>
+          <t>Amlodipin 5 mg</t>
         </is>
       </c>
       <c r="F70" t="n">
         <v>1</v>
       </c>
       <c r="G70" t="n">
-        <v>101</v>
+        <v>74</v>
       </c>
       <c r="H70" t="n">
-        <v>101</v>
+        <v>74</v>
       </c>
     </row>
     <row r="71">
@@ -3736,32 +3736,32 @@
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>P0040</t>
+          <t>P0058</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>Středočeský</t>
+          <t>Praha</t>
         </is>
       </c>
       <c r="D71" t="inlineStr">
         <is>
-          <t>L02</t>
+          <t>L04</t>
         </is>
       </c>
       <c r="E71" t="inlineStr">
         <is>
-          <t>Atorvastatin 20 mg</t>
+          <t>Ramipril 5 mg</t>
         </is>
       </c>
       <c r="F71" t="n">
         <v>1</v>
       </c>
       <c r="G71" t="n">
-        <v>149</v>
+        <v>101</v>
       </c>
       <c r="H71" t="n">
-        <v>149</v>
+        <v>101</v>
       </c>
     </row>
     <row r="72">
@@ -3770,12 +3770,12 @@
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>P0040</t>
+          <t>P0059</t>
         </is>
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>Středočeský</t>
+          <t>Praha</t>
         </is>
       </c>
       <c r="D72" t="inlineStr">
@@ -3804,12 +3804,12 @@
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>P0041</t>
+          <t>P0060</t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>Jihomoravský</t>
+          <t>Moravskoslezský</t>
         </is>
       </c>
       <c r="D73" t="inlineStr">
@@ -3838,7 +3838,7 @@
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>P0041</t>
+          <t>P0061</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
@@ -3848,22 +3848,22 @@
       </c>
       <c r="D74" t="inlineStr">
         <is>
-          <t>L07</t>
+          <t>L05</t>
         </is>
       </c>
       <c r="E74" t="inlineStr">
         <is>
-          <t>Sertralin 50 mg</t>
+          <t>Levothyroxin 50 µg</t>
         </is>
       </c>
       <c r="F74" t="n">
         <v>1</v>
       </c>
       <c r="G74" t="n">
-        <v>215</v>
+        <v>122</v>
       </c>
       <c r="H74" t="n">
-        <v>215</v>
+        <v>122</v>
       </c>
     </row>
     <row r="75">
@@ -3872,32 +3872,32 @@
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>P0042</t>
+          <t>P0061</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>Středočeský</t>
+          <t>Jihomoravský</t>
         </is>
       </c>
       <c r="D75" t="inlineStr">
         <is>
-          <t>L02</t>
+          <t>L07</t>
         </is>
       </c>
       <c r="E75" t="inlineStr">
         <is>
-          <t>Atorvastatin 20 mg</t>
+          <t>Sertralin 50 mg</t>
         </is>
       </c>
       <c r="F75" t="n">
         <v>1</v>
       </c>
       <c r="G75" t="n">
-        <v>149</v>
+        <v>216</v>
       </c>
       <c r="H75" t="n">
-        <v>149</v>
+        <v>216</v>
       </c>
     </row>
     <row r="76">
@@ -3906,32 +3906,32 @@
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>P0043</t>
+          <t>P0061</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>Středočeský</t>
+          <t>Jihomoravský</t>
         </is>
       </c>
       <c r="D76" t="inlineStr">
         <is>
-          <t>L04</t>
+          <t>L09</t>
         </is>
       </c>
       <c r="E76" t="inlineStr">
         <is>
-          <t>Ramipril 5 mg</t>
+          <t>Amoxicilin 500 mg</t>
         </is>
       </c>
       <c r="F76" t="n">
         <v>1</v>
       </c>
       <c r="G76" t="n">
-        <v>101</v>
+        <v>124</v>
       </c>
       <c r="H76" t="n">
-        <v>101</v>
+        <v>124</v>
       </c>
     </row>
     <row r="77">
@@ -3940,12 +3940,12 @@
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>P0044</t>
+          <t>P0062</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>Plzeňský</t>
+          <t>Praha</t>
         </is>
       </c>
       <c r="D77" t="inlineStr">
@@ -3974,32 +3974,32 @@
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>P0044</t>
+          <t>P0062</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>Plzeňský</t>
+          <t>Praha</t>
         </is>
       </c>
       <c r="D78" t="inlineStr">
         <is>
-          <t>L05</t>
+          <t>L06</t>
         </is>
       </c>
       <c r="E78" t="inlineStr">
         <is>
-          <t>Levothyroxin 50 µg</t>
+          <t>Omeprazol 20 mg</t>
         </is>
       </c>
       <c r="F78" t="n">
         <v>1</v>
       </c>
       <c r="G78" t="n">
-        <v>121</v>
+        <v>139</v>
       </c>
       <c r="H78" t="n">
-        <v>121</v>
+        <v>139</v>
       </c>
     </row>
     <row r="79">
@@ -4008,32 +4008,32 @@
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>P0044</t>
+          <t>P0062</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>Plzeňský</t>
+          <t>Praha</t>
         </is>
       </c>
       <c r="D79" t="inlineStr">
         <is>
-          <t>L06</t>
+          <t>L08</t>
         </is>
       </c>
       <c r="E79" t="inlineStr">
         <is>
-          <t>Omeprazol 20 mg</t>
+          <t>Salbutamol inhalátor</t>
         </is>
       </c>
       <c r="F79" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G79" t="n">
-        <v>139</v>
+        <v>170</v>
       </c>
       <c r="H79" t="n">
-        <v>278</v>
+        <v>170</v>
       </c>
     </row>
     <row r="80">
@@ -4042,32 +4042,32 @@
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>P0044</t>
+          <t>P0063</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>Plzeňský</t>
+          <t>Jihomoravský</t>
         </is>
       </c>
       <c r="D80" t="inlineStr">
         <is>
-          <t>L09</t>
+          <t>L04</t>
         </is>
       </c>
       <c r="E80" t="inlineStr">
         <is>
-          <t>Amoxicilin 500 mg</t>
+          <t>Ramipril 5 mg</t>
         </is>
       </c>
       <c r="F80" t="n">
         <v>1</v>
       </c>
       <c r="G80" t="n">
-        <v>124</v>
+        <v>101</v>
       </c>
       <c r="H80" t="n">
-        <v>124</v>
+        <v>101</v>
       </c>
     </row>
     <row r="81">
@@ -4076,7 +4076,7 @@
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>P0045</t>
+          <t>P0064</t>
         </is>
       </c>
       <c r="C81" t="inlineStr">
@@ -4095,13 +4095,13 @@
         </is>
       </c>
       <c r="F81" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G81" t="n">
         <v>101</v>
       </c>
       <c r="H81" t="n">
-        <v>202</v>
+        <v>101</v>
       </c>
     </row>
     <row r="82">
@@ -4110,7 +4110,7 @@
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>P0045</t>
+          <t>P0064</t>
         </is>
       </c>
       <c r="C82" t="inlineStr">
@@ -4132,10 +4132,10 @@
         <v>1</v>
       </c>
       <c r="G82" t="n">
-        <v>215</v>
+        <v>216</v>
       </c>
       <c r="H82" t="n">
-        <v>215</v>
+        <v>216</v>
       </c>
     </row>
     <row r="83">
@@ -4144,32 +4144,32 @@
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>P0046</t>
+          <t>P0064</t>
         </is>
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>Jihomoravský</t>
+          <t>Praha</t>
         </is>
       </c>
       <c r="D83" t="inlineStr">
         <is>
-          <t>L01</t>
+          <t>L08</t>
         </is>
       </c>
       <c r="E83" t="inlineStr">
         <is>
-          <t>Metformin 500 mg</t>
+          <t>Salbutamol inhalátor</t>
         </is>
       </c>
       <c r="F83" t="n">
         <v>1</v>
       </c>
       <c r="G83" t="n">
-        <v>92</v>
+        <v>170</v>
       </c>
       <c r="H83" t="n">
-        <v>92</v>
+        <v>170</v>
       </c>
     </row>
     <row r="84">
@@ -4178,7 +4178,7 @@
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>P0047</t>
+          <t>P0065</t>
         </is>
       </c>
       <c r="C84" t="inlineStr">
@@ -4188,22 +4188,22 @@
       </c>
       <c r="D84" t="inlineStr">
         <is>
-          <t>L03</t>
+          <t>L07</t>
         </is>
       </c>
       <c r="E84" t="inlineStr">
         <is>
-          <t>Amlodipin 5 mg</t>
+          <t>Sertralin 50 mg</t>
         </is>
       </c>
       <c r="F84" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G84" t="n">
-        <v>74</v>
+        <v>216</v>
       </c>
       <c r="H84" t="n">
-        <v>148</v>
+        <v>216</v>
       </c>
     </row>
     <row r="85">
@@ -4212,32 +4212,32 @@
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>P0047</t>
+          <t>P0066</t>
         </is>
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>Jihomoravský</t>
+          <t>Olomoucký</t>
         </is>
       </c>
       <c r="D85" t="inlineStr">
         <is>
-          <t>L07</t>
+          <t>L04</t>
         </is>
       </c>
       <c r="E85" t="inlineStr">
         <is>
-          <t>Sertralin 50 mg</t>
+          <t>Ramipril 5 mg</t>
         </is>
       </c>
       <c r="F85" t="n">
         <v>1</v>
       </c>
       <c r="G85" t="n">
-        <v>215</v>
+        <v>101</v>
       </c>
       <c r="H85" t="n">
-        <v>215</v>
+        <v>101</v>
       </c>
     </row>
     <row r="86">
@@ -4246,32 +4246,32 @@
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>P0048</t>
+          <t>P0066</t>
         </is>
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>Praha</t>
+          <t>Olomoucký</t>
         </is>
       </c>
       <c r="D86" t="inlineStr">
         <is>
-          <t>L01</t>
+          <t>L05</t>
         </is>
       </c>
       <c r="E86" t="inlineStr">
         <is>
-          <t>Metformin 500 mg</t>
+          <t>Levothyroxin 50 µg</t>
         </is>
       </c>
       <c r="F86" t="n">
         <v>2</v>
       </c>
       <c r="G86" t="n">
-        <v>92</v>
+        <v>122</v>
       </c>
       <c r="H86" t="n">
-        <v>184</v>
+        <v>244</v>
       </c>
     </row>
     <row r="87">
@@ -4280,304 +4280,32 @@
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>P0049</t>
+          <t>P0066</t>
         </is>
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>Plzeňský</t>
+          <t>Olomoucký</t>
         </is>
       </c>
       <c r="D87" t="inlineStr">
         <is>
-          <t>L04</t>
+          <t>L09</t>
         </is>
       </c>
       <c r="E87" t="inlineStr">
         <is>
-          <t>Ramipril 5 mg</t>
+          <t>Amoxicilin 500 mg</t>
         </is>
       </c>
       <c r="F87" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G87" t="n">
-        <v>101</v>
+        <v>124</v>
       </c>
       <c r="H87" t="n">
-        <v>202</v>
-      </c>
-    </row>
-    <row r="88">
-      <c r="A88" s="10" t="n">
-        <v>46357</v>
-      </c>
-      <c r="B88" t="inlineStr">
-        <is>
-          <t>P0050</t>
-        </is>
-      </c>
-      <c r="C88" t="inlineStr">
-        <is>
-          <t>Jihomoravský</t>
-        </is>
-      </c>
-      <c r="D88" t="inlineStr">
-        <is>
-          <t>L07</t>
-        </is>
-      </c>
-      <c r="E88" t="inlineStr">
-        <is>
-          <t>Sertralin 50 mg</t>
-        </is>
-      </c>
-      <c r="F88" t="n">
-        <v>1</v>
-      </c>
-      <c r="G88" t="n">
-        <v>215</v>
-      </c>
-      <c r="H88" t="n">
-        <v>215</v>
-      </c>
-    </row>
-    <row r="89">
-      <c r="A89" s="10" t="n">
-        <v>46357</v>
-      </c>
-      <c r="B89" t="inlineStr">
-        <is>
-          <t>P0051</t>
-        </is>
-      </c>
-      <c r="C89" t="inlineStr">
-        <is>
-          <t>Jihomoravský</t>
-        </is>
-      </c>
-      <c r="D89" t="inlineStr">
-        <is>
-          <t>L01</t>
-        </is>
-      </c>
-      <c r="E89" t="inlineStr">
-        <is>
-          <t>Metformin 500 mg</t>
-        </is>
-      </c>
-      <c r="F89" t="n">
-        <v>1</v>
-      </c>
-      <c r="G89" t="n">
-        <v>92</v>
-      </c>
-      <c r="H89" t="n">
-        <v>92</v>
-      </c>
-    </row>
-    <row r="90">
-      <c r="A90" s="10" t="n">
-        <v>46357</v>
-      </c>
-      <c r="B90" t="inlineStr">
-        <is>
-          <t>P0052</t>
-        </is>
-      </c>
-      <c r="C90" t="inlineStr">
-        <is>
-          <t>Středočeský</t>
-        </is>
-      </c>
-      <c r="D90" t="inlineStr">
-        <is>
-          <t>L02</t>
-        </is>
-      </c>
-      <c r="E90" t="inlineStr">
-        <is>
-          <t>Atorvastatin 20 mg</t>
-        </is>
-      </c>
-      <c r="F90" t="n">
-        <v>1</v>
-      </c>
-      <c r="G90" t="n">
-        <v>149</v>
-      </c>
-      <c r="H90" t="n">
-        <v>149</v>
-      </c>
-    </row>
-    <row r="91">
-      <c r="A91" s="10" t="n">
-        <v>46357</v>
-      </c>
-      <c r="B91" t="inlineStr">
-        <is>
-          <t>P0053</t>
-        </is>
-      </c>
-      <c r="C91" t="inlineStr">
-        <is>
-          <t>Středočeský</t>
-        </is>
-      </c>
-      <c r="D91" t="inlineStr">
-        <is>
-          <t>L01</t>
-        </is>
-      </c>
-      <c r="E91" t="inlineStr">
-        <is>
-          <t>Metformin 500 mg</t>
-        </is>
-      </c>
-      <c r="F91" t="n">
-        <v>1</v>
-      </c>
-      <c r="G91" t="n">
-        <v>92</v>
-      </c>
-      <c r="H91" t="n">
-        <v>92</v>
-      </c>
-    </row>
-    <row r="92">
-      <c r="A92" s="10" t="n">
-        <v>46357</v>
-      </c>
-      <c r="B92" t="inlineStr">
-        <is>
-          <t>P0053</t>
-        </is>
-      </c>
-      <c r="C92" t="inlineStr">
-        <is>
-          <t>Středočeský</t>
-        </is>
-      </c>
-      <c r="D92" t="inlineStr">
-        <is>
-          <t>L06</t>
-        </is>
-      </c>
-      <c r="E92" t="inlineStr">
-        <is>
-          <t>Omeprazol 20 mg</t>
-        </is>
-      </c>
-      <c r="F92" t="n">
-        <v>2</v>
-      </c>
-      <c r="G92" t="n">
-        <v>139</v>
-      </c>
-      <c r="H92" t="n">
-        <v>278</v>
-      </c>
-    </row>
-    <row r="93">
-      <c r="A93" s="10" t="n">
-        <v>46357</v>
-      </c>
-      <c r="B93" t="inlineStr">
-        <is>
-          <t>P0054</t>
-        </is>
-      </c>
-      <c r="C93" t="inlineStr">
-        <is>
-          <t>Jihomoravský</t>
-        </is>
-      </c>
-      <c r="D93" t="inlineStr">
-        <is>
-          <t>L02</t>
-        </is>
-      </c>
-      <c r="E93" t="inlineStr">
-        <is>
-          <t>Atorvastatin 20 mg</t>
-        </is>
-      </c>
-      <c r="F93" t="n">
-        <v>1</v>
-      </c>
-      <c r="G93" t="n">
-        <v>149</v>
-      </c>
-      <c r="H93" t="n">
-        <v>149</v>
-      </c>
-    </row>
-    <row r="94">
-      <c r="A94" s="10" t="n">
-        <v>46357</v>
-      </c>
-      <c r="B94" t="inlineStr">
-        <is>
-          <t>P0055</t>
-        </is>
-      </c>
-      <c r="C94" t="inlineStr">
-        <is>
-          <t>Středočeský</t>
-        </is>
-      </c>
-      <c r="D94" t="inlineStr">
-        <is>
-          <t>L02</t>
-        </is>
-      </c>
-      <c r="E94" t="inlineStr">
-        <is>
-          <t>Atorvastatin 20 mg</t>
-        </is>
-      </c>
-      <c r="F94" t="n">
-        <v>1</v>
-      </c>
-      <c r="G94" t="n">
-        <v>149</v>
-      </c>
-      <c r="H94" t="n">
-        <v>149</v>
-      </c>
-    </row>
-    <row r="95">
-      <c r="A95" s="10" t="n">
-        <v>46357</v>
-      </c>
-      <c r="B95" t="inlineStr">
-        <is>
-          <t>P0055</t>
-        </is>
-      </c>
-      <c r="C95" t="inlineStr">
-        <is>
-          <t>Středočeský</t>
-        </is>
-      </c>
-      <c r="D95" t="inlineStr">
-        <is>
-          <t>L05</t>
-        </is>
-      </c>
-      <c r="E95" t="inlineStr">
-        <is>
-          <t>Levothyroxin 50 µg</t>
-        </is>
-      </c>
-      <c r="F95" t="n">
-        <v>1</v>
-      </c>
-      <c r="G95" t="n">
-        <v>121</v>
-      </c>
-      <c r="H95" t="n">
-        <v>121</v>
+        <v>124</v>
       </c>
     </row>
   </sheetData>

</xml_diff>